<commit_message>
feat: multi-monitor, analysis shortcuts and window management fixes
</commit_message>
<xml_diff>
--- a/SAVE/Rapport_Analyse_20260101_20260316.xlsx
+++ b/SAVE/Rapport_Analyse_20260101_20260316.xlsx
@@ -2152,6 +2152,42 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7620000" cy="3810000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="EvolutionChart"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId13" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7620000" cy="3810000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -38273,6 +38309,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
@@ -38906,7 +38943,7 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:tableParts count="1">
-    <x:tablePart r:id="rId12"/>
+    <x:tablePart r:id="rId14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>